<commit_message>
Sprint 6.5: RBAC (Phases 1-5), doc type cloning, CSV/Excel export
- RBAC Phases 1-5: Data model & migration 006, permission engine (single
  chokepoint), route refactoring (23+ endpoints), API key re-scoping,
  frontend RBAC (reviewer→editor, project-level permission map)
- Document type cloning: POST /document-types/{id}/clone endpoint + UI button
- CSV/Excel export: GET /documents/export?format=csv|xlsx + UI Export button
- 107 backend tests pass, 20 frontend tests pass, tsc --noEmit clean
</commit_message>
<xml_diff>
--- a/ActionBridge_Sprint_Planning.xlsx
+++ b/ActionBridge_Sprint_Planning.xlsx
@@ -63,7 +63,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -106,6 +106,12 @@
         <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -133,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -180,6 +186,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -574,6 +586,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2755,19 +2768,19 @@
       </c>
     </row>
     <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="11" t="inlineStr">
+      <c r="A66" s="18" t="inlineStr">
         <is>
           <t>S6.1</t>
         </is>
       </c>
-      <c r="B66" s="11" t="inlineStr">
+      <c r="B66" s="18" t="inlineStr">
         <is>
           <t>Backend: pytest setup + conftest (test DB, auth fixtures)</t>
         </is>
       </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D66" s="14" t="inlineStr">
@@ -2789,19 +2802,19 @@
       <c r="H66" s="11" t="inlineStr"/>
     </row>
     <row r="67" ht="22" customHeight="1">
-      <c r="A67" s="11" t="inlineStr">
+      <c r="A67" s="18" t="inlineStr">
         <is>
           <t>S6.2</t>
         </is>
       </c>
-      <c r="B67" s="11" t="inlineStr">
+      <c r="B67" s="18" t="inlineStr">
         <is>
           <t>Backend: test auth endpoints (login, register, setup, me, users)</t>
         </is>
       </c>
-      <c r="C67" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D67" s="14" t="inlineStr">
@@ -2823,19 +2836,19 @@
       <c r="H67" s="11" t="inlineStr"/>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="11" t="inlineStr">
+      <c r="A68" s="18" t="inlineStr">
         <is>
           <t>S6.3</t>
         </is>
       </c>
-      <c r="B68" s="11" t="inlineStr">
+      <c r="B68" s="18" t="inlineStr">
         <is>
           <t>Backend: test project CRUD + member invite/accept/remove</t>
         </is>
       </c>
-      <c r="C68" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C68" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D68" s="14" t="inlineStr">
@@ -2857,19 +2870,19 @@
       <c r="H68" s="11" t="inlineStr"/>
     </row>
     <row r="69" ht="22" customHeight="1">
-      <c r="A69" s="11" t="inlineStr">
+      <c r="A69" s="18" t="inlineStr">
         <is>
           <t>S6.4</t>
         </is>
       </c>
-      <c r="B69" s="11" t="inlineStr">
+      <c r="B69" s="18" t="inlineStr">
         <is>
           <t>Backend: test document submission, validation rules, FSM transitions</t>
         </is>
       </c>
-      <c r="C69" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D69" s="14" t="inlineStr">
@@ -2891,19 +2904,19 @@
       <c r="H69" s="11" t="inlineStr"/>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
+      <c r="A70" s="18" t="inlineStr">
         <is>
           <t>S6.5</t>
         </is>
       </c>
-      <c r="B70" s="11" t="inlineStr">
+      <c r="B70" s="18" t="inlineStr">
         <is>
           <t>Backend: test comments, attachments, notifications, subscriptions</t>
         </is>
       </c>
-      <c r="C70" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C70" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D70" s="12" t="inlineStr">
@@ -2925,19 +2938,19 @@
       <c r="H70" s="11" t="inlineStr"/>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="11" t="inlineStr">
+      <c r="A71" s="18" t="inlineStr">
         <is>
           <t>S6.6</t>
         </is>
       </c>
-      <c r="B71" s="11" t="inlineStr">
+      <c r="B71" s="18" t="inlineStr">
         <is>
           <t>Backend: test regex-patterns CRUD + pattern resolution in validation</t>
         </is>
       </c>
-      <c r="C71" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D71" s="12" t="inlineStr">
@@ -2959,19 +2972,19 @@
       <c r="H71" s="11" t="inlineStr"/>
     </row>
     <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="11" t="inlineStr">
+      <c r="A72" s="18" t="inlineStr">
         <is>
           <t>S6.7</t>
         </is>
       </c>
-      <c r="B72" s="11" t="inlineStr">
+      <c r="B72" s="18" t="inlineStr">
         <is>
           <t>Frontend: vitest + testing-library setup</t>
         </is>
       </c>
-      <c r="C72" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D72" s="12" t="inlineStr">
@@ -2993,19 +3006,19 @@
       <c r="H72" s="11" t="inlineStr"/>
     </row>
     <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="11" t="inlineStr">
+      <c r="A73" s="18" t="inlineStr">
         <is>
           <t>S6.8</t>
         </is>
       </c>
-      <c r="B73" s="11" t="inlineStr">
+      <c r="B73" s="18" t="inlineStr">
         <is>
           <t>Frontend: test schema builder, validation rules dialog, regex builder</t>
         </is>
       </c>
-      <c r="C73" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -3027,19 +3040,19 @@
       <c r="H73" s="11" t="inlineStr"/>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="11" t="inlineStr">
+      <c r="A74" s="18" t="inlineStr">
         <is>
           <t>S6.9</t>
         </is>
       </c>
-      <c r="B74" s="11" t="inlineStr">
+      <c r="B74" s="18" t="inlineStr">
         <is>
           <t>Frontend: test auth flow (login, setup, password reset)</t>
         </is>
       </c>
-      <c r="C74" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C74" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D74" s="12" t="inlineStr">
@@ -3891,20 +3904,21 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3929,19 +3943,19 @@
       </c>
     </row>
     <row r="5" ht="55" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Backend: pytest + httpx + test DB setup</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -3966,19 +3980,19 @@
       </c>
     </row>
     <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Backend: test auth endpoints</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -3999,19 +4013,19 @@
       <c r="G6" s="11" t="inlineStr"/>
     </row>
     <row r="7" ht="55" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Backend: test project + membership</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -4032,19 +4046,19 @@
       <c r="G7" s="11" t="inlineStr"/>
     </row>
     <row r="8" ht="55" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Backend: test document + validation</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -4065,19 +4079,19 @@
       <c r="G8" s="11" t="inlineStr"/>
     </row>
     <row r="9" ht="55" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Backend: test new routers (comments, attachments, notifications, subscriptions)</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -4098,19 +4112,19 @@
       <c r="G9" s="11" t="inlineStr"/>
     </row>
     <row r="10" ht="55" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Frontend: vitest + testing-library setup</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -4131,19 +4145,19 @@
       <c r="G10" s="11" t="inlineStr"/>
     </row>
     <row r="11" ht="55" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Frontend: test SchemaBuilder + ValidationRulesDialog</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -4168,19 +4182,19 @@
       </c>
     </row>
     <row r="12" ht="55" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Frontend: test auth flow</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">

</xml_diff>